<commit_message>
validate "Column definitions" worksheet
- vmr_export:
    - Add strict validation for `Column definitions` against VMR headers up to
      `Editor Notes`.
    - Validate grouped `D - R` taxonomy header coverage (`Realm`..`Species`).
    - Validate controlled-value definitions by checking every `Column Values`
      entry appears in `Definition` bullet lists.
    - Add `-k/--keep-going` to downgrade Column Definitions mismatches to warnings
      and continue; default behavior fails after full validation pass.
    - Keep full issue aggregation before fail/continue decision.

- Makefile:
    - Add --keep-going flag to vmr_export.py
</commit_message>
<xml_diff>
--- a/test_data/export/expected-errors.xlsx
+++ b/test_data/export/expected-errors.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="errors" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="errors" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B66"/>
+  <dimension ref="A1:B73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -707,96 +707,96 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>INFO</t>
+          <t>WARNING</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Read 17916 rows from file test_data/export/ICTVdatabase/data/vmr_export.utf8.txt</t>
+          <t>Worksheet 'Column definitions' is missing documentation for VMR header 'Host source' from worksheet 'VMR MSL40'</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>SUCCESS</t>
+          <t>WARNING</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Column match: 'Isolate ID'</t>
+          <t>Worksheet 'Column definitions' Definition for 'Genome coverage' is missing value 'Not Compliant' from worksheet 'Column Values'</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>SUCCESS</t>
+          <t>WARNING</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Column match: 'Species Sort'</t>
+          <t>Worksheet 'Column definitions' Definition for 'Genome' is missing value 'dsDNA; ssDNA' from worksheet 'Column Values'</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>SUCCESS</t>
+          <t>WARNING</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Column match: 'Isolate Sort'</t>
+          <t>Worksheet 'Column definitions' Definition for 'Genome' is missing value 'dsRNA' from worksheet 'Column Values'</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>SUCCESS</t>
+          <t>WARNING</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Column match: 'Realm'</t>
+          <t>Worksheet 'Column definitions' Definition for 'Genome' is missing value 'Unassigned' from worksheet 'Column Values'</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>SUCCESS</t>
+          <t>WARNING</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Column match: 'Subrealm'</t>
+          <t>Worksheet 'Column definitions' Definition for 'Genome' is missing value 'Viroid' from worksheet 'Column Values'</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>SUCCESS</t>
+          <t>WARNING</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Column match: 'Kingdom'</t>
+          <t>Worksheet 'Column definitions' has no Definition text for controlled-value header 'Host source'</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>SUCCESS</t>
+          <t>INFO</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Column match: 'Subkingdom'</t>
+          <t>Read 17916 rows from file test_data/export/ICTVdatabase/data/vmr_export.utf8.txt</t>
         </is>
       </c>
     </row>
@@ -808,7 +808,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Column match: 'Phylum'</t>
+          <t>Column match: 'Isolate ID'</t>
         </is>
       </c>
     </row>
@@ -820,7 +820,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Column match: 'Subphylum'</t>
+          <t>Column match: 'Species Sort'</t>
         </is>
       </c>
     </row>
@@ -832,7 +832,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Column match: 'Class'</t>
+          <t>Column match: 'Isolate Sort'</t>
         </is>
       </c>
     </row>
@@ -844,7 +844,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Column match: 'Subclass'</t>
+          <t>Column match: 'Realm'</t>
         </is>
       </c>
     </row>
@@ -856,7 +856,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Column match: 'Order'</t>
+          <t>Column match: 'Subrealm'</t>
         </is>
       </c>
     </row>
@@ -868,7 +868,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Column match: 'Suborder'</t>
+          <t>Column match: 'Kingdom'</t>
         </is>
       </c>
     </row>
@@ -880,7 +880,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Column match: 'Family'</t>
+          <t>Column match: 'Subkingdom'</t>
         </is>
       </c>
     </row>
@@ -892,7 +892,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Column match: 'Subfamily'</t>
+          <t>Column match: 'Phylum'</t>
         </is>
       </c>
     </row>
@@ -904,7 +904,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Column match: 'Genus'</t>
+          <t>Column match: 'Subphylum'</t>
         </is>
       </c>
     </row>
@@ -916,7 +916,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Column match: 'Subgenus'</t>
+          <t>Column match: 'Class'</t>
         </is>
       </c>
     </row>
@@ -928,7 +928,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Column match: 'Species'</t>
+          <t>Column match: 'Subclass'</t>
         </is>
       </c>
     </row>
@@ -940,7 +940,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Column match: 'ICTV_ID'</t>
+          <t>Column match: 'Order'</t>
         </is>
       </c>
     </row>
@@ -952,7 +952,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Column match: 'Exemplar or additional isolate'</t>
+          <t>Column match: 'Suborder'</t>
         </is>
       </c>
     </row>
@@ -964,7 +964,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Column match: 'Virus name(s)'</t>
+          <t>Column match: 'Family'</t>
         </is>
       </c>
     </row>
@@ -976,7 +976,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Column match: 'Virus name abbreviation(s)'</t>
+          <t>Column match: 'Subfamily'</t>
         </is>
       </c>
     </row>
@@ -988,7 +988,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Column match: 'Virus isolate designation'</t>
+          <t>Column match: 'Genus'</t>
         </is>
       </c>
     </row>
@@ -1000,7 +1000,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Column match: 'Virus GENBANK accession'</t>
+          <t>Column match: 'Subgenus'</t>
         </is>
       </c>
     </row>
@@ -1012,7 +1012,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Column match: 'Genome coverage'</t>
+          <t>Column match: 'Species'</t>
         </is>
       </c>
     </row>
@@ -1024,7 +1024,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Column match: 'Genome'</t>
+          <t>Column match: 'ICTV_ID'</t>
         </is>
       </c>
     </row>
@@ -1036,7 +1036,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Column match: 'Host source'</t>
+          <t>Column match: 'Exemplar or additional isolate'</t>
         </is>
       </c>
     </row>
@@ -1048,7 +1048,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Column match: 'Accessions Link'</t>
+          <t>Column match: 'Virus name(s)'</t>
         </is>
       </c>
     </row>
@@ -1060,7 +1060,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Column match: 'Editor Notes'</t>
+          <t>Column match: 'Virus name abbreviation(s)'</t>
         </is>
       </c>
     </row>
@@ -1072,7 +1072,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Column match: 'QC_status'</t>
+          <t>Column match: 'Virus isolate designation'</t>
         </is>
       </c>
     </row>
@@ -1084,7 +1084,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Column match: 'QC_taxon_inher_molecule'</t>
+          <t>Column match: 'Virus GENBANK accession'</t>
         </is>
       </c>
     </row>
@@ -1096,7 +1096,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Column match: 'QC_taxon_change'</t>
+          <t>Column match: 'Genome coverage'</t>
         </is>
       </c>
     </row>
@@ -1108,91 +1108,91 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Column match: 'QC_taxon_proposal'</t>
+          <t>Column match: 'Genome'</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>INFO</t>
+          <t>SUCCESS</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Populating Original worksheet</t>
+          <t>Column match: 'Host source'</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>INFO</t>
+          <t>SUCCESS</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Wrote 17916 rows into worksheet 'Original'</t>
+          <t>Column match: 'Accessions Link'</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>INFO</t>
+          <t>SUCCESS</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Populating VMR MSL40 worksheet</t>
+          <t>Column match: 'Editor Notes'</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>INFO</t>
+          <t>SUCCESS</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Wrote 17916 rows into worksheet 'VMR MSL40'</t>
+          <t>Column match: 'QC_status'</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>INFO</t>
+          <t>SUCCESS</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Added 17916 isolate hyperlinks in worksheet 'VMR MSL40'</t>
+          <t>Column match: 'QC_taxon_inher_molecule'</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>INFO</t>
+          <t>SUCCESS</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Read 40 rows from file test_data/export/ICTVdatabase/data/taxonomy_toc.utf8.txt</t>
+          <t>Column match: 'QC_taxon_change'</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>INFO</t>
+          <t>SUCCESS</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Wrote workbook with 8 worksheet(s) to test_out/export/VMR.editor.xlsx</t>
+          <t>Column match: 'QC_taxon_proposal'</t>
         </is>
       </c>
     </row>
@@ -1203,6 +1203,90 @@
         </is>
       </c>
       <c r="B66" t="inlineStr">
+        <is>
+          <t>Populating Original worksheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Wrote 17916 rows into worksheet 'Original'</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Populating VMR MSL40 worksheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Wrote 17916 rows into worksheet 'VMR MSL40'</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Added 17916 isolate hyperlinks in worksheet 'VMR MSL40'</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Read 40 rows from file test_data/export/ICTVdatabase/data/taxonomy_toc.utf8.txt</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Wrote workbook with 8 worksheet(s) to test_out/export/VMR.editor.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
         <is>
           <t>Wrote 4 worksheet(s) to public file test_out/export/VMR.xlsx</t>
         </is>

</xml_diff>

<commit_message>
add -mask db_mask.tsv to remove values from db before building export
Specifically, we're blocking genome_molecule of ['Viroid' and 'Unassigned'], which are historical, and no longer used/allowed.
</commit_message>
<xml_diff>
--- a/test_data/export/expected-errors.xlsx
+++ b/test_data/export/expected-errors.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B73"/>
+  <dimension ref="A1:B160"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -436,19 +436,19 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Read template workbook from test_data/export/VMR_MSL40.v2.20251013.editor.hacked.xlsx</t>
+          <t>Loaded 2 mask rule(s) from test_data/export/db_mask.tsv</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>SUCCESS</t>
+          <t>INFO</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Validated worksheet: Version</t>
+          <t>Read template workbook from test_data/export/VMR_MSL40.v2.20251013.editor.hacked.xlsx</t>
         </is>
       </c>
     </row>
@@ -460,7 +460,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Validated worksheet: VMR MSL40</t>
+          <t>Validated worksheet: Version</t>
         </is>
       </c>
     </row>
@@ -472,7 +472,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Validated worksheet: Column definitions</t>
+          <t>Validated worksheet: VMR MSL40</t>
         </is>
       </c>
     </row>
@@ -484,7 +484,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Validated worksheet: Column Values</t>
+          <t>Validated worksheet: Column definitions</t>
         </is>
       </c>
     </row>
@@ -496,7 +496,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Validated worksheet: README.editor</t>
+          <t>Validated worksheet: Column Values</t>
         </is>
       </c>
     </row>
@@ -508,7 +508,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Validated worksheet: CHANGELOG.editor</t>
+          <t>Validated worksheet: README.editor</t>
         </is>
       </c>
     </row>
@@ -520,7 +520,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Validated worksheet: Original</t>
+          <t>Validated worksheet: CHANGELOG.editor</t>
         </is>
       </c>
     </row>
@@ -532,19 +532,19 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Validated worksheet: Original Column Values</t>
+          <t>Validated worksheet: Original</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>INFO</t>
+          <t>SUCCESS</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Wrote 2 values to sheet 'Original Column Values' column 'Exemplar or additional isolate'</t>
+          <t>Validated worksheet: Original Column Values</t>
         </is>
       </c>
     </row>
@@ -556,7 +556,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Read 5 rows from file test_data/export/ICTVdatabase/data/taxonomy_genome_coverage.utf8.txt</t>
+          <t>Wrote 2 values to sheet 'Original Column Values' column 'Exemplar or additional isolate'</t>
         </is>
       </c>
     </row>
@@ -568,7 +568,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Wrote 5 values to sheet 'Original Column Values' column 'Genome coverage'</t>
+          <t>Read 5 rows from file test_data/export/ICTVdatabase/data/taxonomy_genome_coverage.utf8.txt</t>
         </is>
       </c>
     </row>
@@ -580,7 +580,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Read 16 rows from file test_data/export/ICTVdatabase/data/taxonomy_molecule.utf8.txt</t>
+          <t>Wrote 5 values to sheet 'Original Column Values' column 'Genome coverage'</t>
         </is>
       </c>
     </row>
@@ -592,7 +592,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Wrote 16 values to sheet 'Original Column Values' column 'Genome'</t>
+          <t>Applied 2 flatfile mask rule(s) to table 'taxonomy_molecule'</t>
         </is>
       </c>
     </row>
@@ -604,7 +604,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Read 27 rows from file test_data/export/ICTVdatabase/data/taxonomy_host_source.utf8.txt</t>
+          <t>Read 14 rows from file test_data/export/ICTVdatabase/data/taxonomy_molecule.utf8.txt</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Wrote 27 values to sheet 'Original Column Values' column 'Host source'</t>
+          <t>Wrote 14 values to sheet 'Original Column Values' column 'Genome'</t>
         </is>
       </c>
     </row>
@@ -628,7 +628,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Wrote 2 values to sheet 'Column Values' column 'Exemplar or additional isolate'</t>
+          <t>Read 27 rows from file test_data/export/ICTVdatabase/data/taxonomy_host_source.utf8.txt</t>
         </is>
       </c>
     </row>
@@ -640,7 +640,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Read 5 rows from file test_data/export/ICTVdatabase/data/taxonomy_genome_coverage.utf8.txt</t>
+          <t>Wrote 27 values to sheet 'Original Column Values' column 'Host source'</t>
         </is>
       </c>
     </row>
@@ -652,7 +652,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Wrote 5 values to sheet 'Column Values' column 'Genome coverage'</t>
+          <t>Wrote 2 values to sheet 'Column Values' column 'Exemplar or additional isolate'</t>
         </is>
       </c>
     </row>
@@ -664,7 +664,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Read 16 rows from file test_data/export/ICTVdatabase/data/taxonomy_molecule.utf8.txt</t>
+          <t>Read 5 rows from file test_data/export/ICTVdatabase/data/taxonomy_genome_coverage.utf8.txt</t>
         </is>
       </c>
     </row>
@@ -676,7 +676,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Wrote 16 values to sheet 'Column Values' column 'Genome'</t>
+          <t>Wrote 5 values to sheet 'Column Values' column 'Genome coverage'</t>
         </is>
       </c>
     </row>
@@ -688,7 +688,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Read 27 rows from file test_data/export/ICTVdatabase/data/taxonomy_host_source.utf8.txt</t>
+          <t>Applied 2 flatfile mask rule(s) to table 'taxonomy_molecule'</t>
         </is>
       </c>
     </row>
@@ -700,91 +700,91 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Wrote 27 values to sheet 'Column Values' column 'Host source'</t>
+          <t>Read 14 rows from file test_data/export/ICTVdatabase/data/taxonomy_molecule.utf8.txt</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>WARNING</t>
+          <t>INFO</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Worksheet 'Column definitions' is missing documentation for VMR header 'Host source' from worksheet 'VMR MSL40'</t>
+          <t>Wrote 14 values to sheet 'Column Values' column 'Genome'</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>WARNING</t>
+          <t>INFO</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Worksheet 'Column definitions' Definition for 'Genome coverage' is missing value 'Not Compliant' from worksheet 'Column Values'</t>
+          <t>Read 27 rows from file test_data/export/ICTVdatabase/data/taxonomy_host_source.utf8.txt</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>WARNING</t>
+          <t>INFO</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Worksheet 'Column definitions' Definition for 'Genome' is missing value 'dsDNA; ssDNA' from worksheet 'Column Values'</t>
+          <t>Wrote 27 values to sheet 'Column Values' column 'Host source'</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>WARNING</t>
+          <t>INFO</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Worksheet 'Column definitions' Definition for 'Genome' is missing value 'dsRNA' from worksheet 'Column Values'</t>
+          <t>Header map: VMR 'Isolate ID' -&gt; Defs 'Isolate ID'</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>WARNING</t>
+          <t>INFO</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Worksheet 'Column definitions' Definition for 'Genome' is missing value 'Unassigned' from worksheet 'Column Values'</t>
+          <t>Header map: VMR 'Species Sort' -&gt; Defs 'Species Sort'</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>WARNING</t>
+          <t>INFO</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Worksheet 'Column definitions' Definition for 'Genome' is missing value 'Viroid' from worksheet 'Column Values'</t>
+          <t>Header map: VMR 'Isolate Sort' -&gt; Defs 'Isolate Sort'</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>WARNING</t>
+          <t>INFO</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Worksheet 'Column definitions' has no Definition text for controlled-value header 'Host source'</t>
+          <t>Header map: VMR 'Realm' -&gt; Defs 'Realm'</t>
         </is>
       </c>
     </row>
@@ -796,403 +796,403 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Read 17916 rows from file test_data/export/ICTVdatabase/data/vmr_export.utf8.txt</t>
+          <t>Header map: VMR 'Subrealm' -&gt; Defs 'Subrealm'</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>SUCCESS</t>
+          <t>INFO</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Column match: 'Isolate ID'</t>
+          <t>Header map: VMR 'Kingdom' -&gt; Defs 'Kingdom'</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>SUCCESS</t>
+          <t>INFO</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Column match: 'Species Sort'</t>
+          <t>Header map: VMR 'Subkingdom' -&gt; Defs 'Subkingdom'</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>SUCCESS</t>
+          <t>INFO</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Column match: 'Isolate Sort'</t>
+          <t>Header map: VMR 'Phylum' -&gt; Defs 'Phylum'</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>SUCCESS</t>
+          <t>INFO</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Column match: 'Realm'</t>
+          <t>Header map: VMR 'Subphylum' -&gt; Defs 'Subphylum'</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>SUCCESS</t>
+          <t>INFO</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Column match: 'Subrealm'</t>
+          <t>Header map: VMR 'Class' -&gt; Defs 'Class'</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>SUCCESS</t>
+          <t>INFO</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Column match: 'Kingdom'</t>
+          <t>Header map: VMR 'Subclass' -&gt; Defs 'Subclass'</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>SUCCESS</t>
+          <t>INFO</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Column match: 'Subkingdom'</t>
+          <t>Header map: VMR 'Order' -&gt; Defs 'Order'</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>SUCCESS</t>
+          <t>INFO</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Column match: 'Phylum'</t>
+          <t>Header map: VMR 'Suborder' -&gt; Defs 'Suborder'</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>SUCCESS</t>
+          <t>INFO</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Column match: 'Subphylum'</t>
+          <t>Header map: VMR 'Family' -&gt; Defs 'Family'</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>SUCCESS</t>
+          <t>INFO</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Column match: 'Class'</t>
+          <t>Header map: VMR 'Subfamily' -&gt; Defs 'Subfamily'</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>SUCCESS</t>
+          <t>INFO</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Column match: 'Subclass'</t>
+          <t>Header map: VMR 'Genus' -&gt; Defs 'Genus'</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>SUCCESS</t>
+          <t>INFO</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Column match: 'Order'</t>
+          <t>Header map: VMR 'Subgenus' -&gt; Defs 'Subgenus'</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>SUCCESS</t>
+          <t>INFO</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Column match: 'Suborder'</t>
+          <t>Header map: VMR 'Species' -&gt; Defs 'Species'</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>SUCCESS</t>
+          <t>INFO</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Column match: 'Family'</t>
+          <t>Header map: VMR 'ICTV_ID' -&gt; Defs 'ICTV_ID'</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>SUCCESS</t>
+          <t>INFO</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Column match: 'Subfamily'</t>
+          <t>Header map: VMR 'Exemplar or additional isolate' -&gt; Defs 'Exemplar or additional isolate'</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>SUCCESS</t>
+          <t>INFO</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Column match: 'Genus'</t>
+          <t>Header map: VMR 'Virus name(s)' -&gt; Defs 'Virus name(s)'</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>SUCCESS</t>
+          <t>INFO</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Column match: 'Subgenus'</t>
+          <t>Header map: VMR 'Virus name abbreviation(s)' -&gt; Defs 'Virus name abbreviation(s)'</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>SUCCESS</t>
+          <t>INFO</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Column match: 'Species'</t>
+          <t>Header map: VMR 'Virus isolate designation' -&gt; Defs 'Virus isolate designation'</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>SUCCESS</t>
+          <t>INFO</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Column match: 'ICTV_ID'</t>
+          <t>Header map: VMR 'Virus GENBANK accession' -&gt; Defs 'Virus GENBANK accession'</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>SUCCESS</t>
+          <t>INFO</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Column match: 'Exemplar or additional isolate'</t>
+          <t>Header map: VMR 'Genome coverage' -&gt; Defs 'Genome coverage'</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>SUCCESS</t>
+          <t>INFO</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Column match: 'Virus name(s)'</t>
+          <t>Header map: VMR 'Genome' -&gt; Defs 'Genome'</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>SUCCESS</t>
+          <t>INFO</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Column match: 'Virus name abbreviation(s)'</t>
+          <t>Header map: VMR 'Host source' -&gt; Defs 'Host/Source' (normalized match; text differs)</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>SUCCESS</t>
+          <t>INFO</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Column match: 'Virus isolate designation'</t>
+          <t>Header map: VMR 'Accessions Link' -&gt; Defs 'Accessions Link'</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>SUCCESS</t>
+          <t>INFO</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Column match: 'Virus GENBANK accession'</t>
+          <t>D-R map: VMR 'Realm' -&gt; Defs 'Realm'</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>SUCCESS</t>
+          <t>INFO</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Column match: 'Genome coverage'</t>
+          <t>D-R map: VMR 'Subrealm' -&gt; Defs 'Subrealm'</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>SUCCESS</t>
+          <t>INFO</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Column match: 'Genome'</t>
+          <t>D-R map: VMR 'Kingdom' -&gt; Defs 'Kingdom'</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>SUCCESS</t>
+          <t>INFO</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Column match: 'Host source'</t>
+          <t>D-R map: VMR 'Subkingdom' -&gt; Defs 'Subkingdom'</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>SUCCESS</t>
+          <t>INFO</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Column match: 'Accessions Link'</t>
+          <t>D-R map: VMR 'Phylum' -&gt; Defs 'Phylum'</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>SUCCESS</t>
+          <t>INFO</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Column match: 'Editor Notes'</t>
+          <t>D-R map: VMR 'Subphylum' -&gt; Defs 'Subphylum'</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>SUCCESS</t>
+          <t>INFO</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Column match: 'QC_status'</t>
+          <t>D-R map: VMR 'Class' -&gt; Defs 'Class'</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>SUCCESS</t>
+          <t>INFO</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Column match: 'QC_taxon_inher_molecule'</t>
+          <t>D-R map: VMR 'Subclass' -&gt; Defs 'Subclass'</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>SUCCESS</t>
+          <t>INFO</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Column match: 'QC_taxon_change'</t>
+          <t>D-R map: VMR 'Order' -&gt; Defs 'Order'</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>SUCCESS</t>
+          <t>INFO</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Column match: 'QC_taxon_proposal'</t>
+          <t>D-R map: VMR 'Suborder' -&gt; Defs 'Suborder'</t>
         </is>
       </c>
     </row>
@@ -1204,7 +1204,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Populating Original worksheet</t>
+          <t>D-R map: VMR 'Family' -&gt; Defs 'Family'</t>
         </is>
       </c>
     </row>
@@ -1216,7 +1216,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Wrote 17916 rows into worksheet 'Original'</t>
+          <t>D-R map: VMR 'Subfamily' -&gt; Defs 'Subfamily'</t>
         </is>
       </c>
     </row>
@@ -1228,7 +1228,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Populating VMR MSL40 worksheet</t>
+          <t>D-R map: VMR 'Genus' -&gt; Defs 'Genus'</t>
         </is>
       </c>
     </row>
@@ -1240,7 +1240,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Wrote 17916 rows into worksheet 'VMR MSL40'</t>
+          <t>D-R map: VMR 'Subgenus' -&gt; Defs 'Subgenus'</t>
         </is>
       </c>
     </row>
@@ -1252,7 +1252,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Added 17916 isolate hyperlinks in worksheet 'VMR MSL40'</t>
+          <t>D-R map: VMR 'Species' -&gt; Defs 'Species'</t>
         </is>
       </c>
     </row>
@@ -1264,7 +1264,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Read 40 rows from file test_data/export/ICTVdatabase/data/taxonomy_toc.utf8.txt</t>
+          <t>Value map [Exemplar or additional isolate]: Column Values 'E' -&gt; Definition text match (normalized substring)</t>
         </is>
       </c>
     </row>
@@ -1276,7 +1276,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Wrote workbook with 8 worksheet(s) to test_out/export/VMR.editor.xlsx</t>
+          <t>Value map [Exemplar or additional isolate]: Column Values 'A' -&gt; Definition text match (normalized substring)</t>
         </is>
       </c>
     </row>
@@ -1287,6 +1287,1050 @@
         </is>
       </c>
       <c r="B73" t="inlineStr">
+        <is>
+          <t>Value map [Genome coverage]: Column Values 'Coding-complete genome' -&gt; Definition 'Coding-complete genome'</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Value map [Genome coverage]: Column Values 'Complete genome' -&gt; Definition 'Complete genome'</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Value map [Genome coverage]: Column Values 'No entry in Genbank' -&gt; Definition 'No entry in Genbank'</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Value map [Genome coverage]: Column Values 'Partial genome' -&gt; Definition 'Partial genome'</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Value map [Genome]: Column Values 'dsDNA' -&gt; Definition 'dsDNA'</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Value map [Genome]: Column Values 'dsDNA-RT' -&gt; Definition 'dsDNA-RT'</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Value map [Genome]: Column Values 'ssDNA' -&gt; Definition 'ssDNA'</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Value map [Genome]: Column Values 'ssDNA(+)' -&gt; Definition 'ssDNA(+)'</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Value map [Genome]: Column Values 'ssDNA(+/-)' -&gt; Definition 'ssDNA(+/-)'</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Value map [Genome]: Column Values 'ssDNA(-)' -&gt; Definition 'ssDNA(-)'</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Value map [Genome]: Column Values 'ssRNA' -&gt; Definition 'ssRNA'</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Value map [Genome]: Column Values 'ssRNA(+)' -&gt; Definition 'ssRNA(+)'</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Value map [Genome]: Column Values 'ssRNA(+/-)' -&gt; Definition 'ssRNA(+/-)'</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>Value map [Genome]: Column Values 'ssRNA(-)' -&gt; Definition 'ssRNA(-)'</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Value map [Genome]: Column Values 'ssRNA(-); ssRNA(+/-)' -&gt; Definition 'ssRNA(-); ssRNA(+/-)'</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Value map [Genome]: Column Values 'ssRNA-RT' -&gt; Definition 'ssRNA-RT'</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Value map [Host source]: Column Values 'air (S)' -&gt; Definition 'air (S)'</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Value map [Host source]: Column Values 'archaea' -&gt; Definition 'archaea'</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Value map [Host source]: Column Values 'bacteria' -&gt; Definition 'bacteria'</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>Value map [Host source]: Column Values 'freshwater (S)' -&gt; Definition 'freshwater (S)'</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>Value map [Host source]: Column Values 'fungi' -&gt; Definition 'fungi'</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>Value map [Host source]: Column Values 'invertebrates' -&gt; Definition 'invertebrates'</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>Value map [Host source]: Column Values 'marine (S)' -&gt; Definition 'marine (S)'</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>Value map [Host source]: Column Values 'phytobiome (S)' -&gt; Definition 'phytobiome (S)'</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>Value map [Host source]: Column Values 'plants' -&gt; Definition 'plants'</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>Value map [Host source]: Column Values 'protists' -&gt; Definition 'protists'</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>Value map [Host source]: Column Values 'sewage (S)' -&gt; Definition 'sewage (S)'</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>Value map [Host source]: Column Values 'soil (S)' -&gt; Definition 'soil (S)'</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>Value map [Host source]: Column Values 'unknown (S)' -&gt; Definition 'unknown (S)'</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>Value map [Host source]: Column Values 'vertebrates' -&gt; Definition 'vertebrates'</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>Worksheet 'Column definitions' Definition for 'Genome coverage' is missing value 'Not Compliant' from worksheet 'Column Values'</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>Worksheet 'Column definitions' Definition for 'Genome' is missing value 'dsDNA; ssDNA' from worksheet 'Column Values'</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>Worksheet 'Column definitions' Definition for 'Genome' is missing value 'dsRNA' from worksheet 'Column Values'</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>Worksheet 'Column definitions' Definition for 'Host source' is missing value 'algae' from worksheet 'Column Values'</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>Worksheet 'Column definitions' Definition for 'Host source' is missing value 'bacteria, invertebrates (S)' from worksheet 'Column Values'</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>Worksheet 'Column definitions' Definition for 'Host source' is missing value 'bacteria, vertebrates (S)' from worksheet 'Column Values'</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>Worksheet 'Column definitions' Definition for 'Host source' is missing value 'fungi (S)' from worksheet 'Column Values'</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>Worksheet 'Column definitions' Definition for 'Host source' is missing value 'invertebrates (S)' from worksheet 'Column Values'</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>Worksheet 'Column definitions' Definition for 'Host source' is missing value 'invertebrates, plants' from worksheet 'Column Values'</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>Worksheet 'Column definitions' Definition for 'Host source' is missing value 'invertebrates, vertebrates' from worksheet 'Column Values'</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>Worksheet 'Column definitions' Definition for 'Host source' is missing value 'oomycetes' from worksheet 'Column Values'</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>Worksheet 'Column definitions' Definition for 'Host source' is missing value 'other (specify)' from worksheet 'Column Values'</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>Worksheet 'Column definitions' Definition for 'Host source' is missing value 'plants (S)' from worksheet 'Column Values'</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>Worksheet 'Column definitions' Definition for 'Host source' is missing value 'plants, fungi' from worksheet 'Column Values'</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>Worksheet 'Column definitions' Definition for 'Host source' is missing value 'protists (S)' from worksheet 'Column Values'</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>Worksheet 'Column definitions' Definition for 'Host source' is missing value 'vertebrates (S)' from worksheet 'Column Values'</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>Read 17916 rows from file test_data/export/ICTVdatabase/data/vmr_export.utf8.txt</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>Column match: 'Isolate ID'</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>Column match: 'Species Sort'</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>Column match: 'Isolate Sort'</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>Column match: 'Realm'</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>Column match: 'Subrealm'</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>Column match: 'Kingdom'</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>Column match: 'Subkingdom'</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>Column match: 'Phylum'</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>Column match: 'Subphylum'</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>Column match: 'Class'</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>Column match: 'Subclass'</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>Column match: 'Order'</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>Column match: 'Suborder'</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>Column match: 'Family'</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>Column match: 'Subfamily'</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>Column match: 'Genus'</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>Column match: 'Subgenus'</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>Column match: 'Species'</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>Column match: 'ICTV_ID'</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>Column match: 'Exemplar or additional isolate'</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>Column match: 'Virus name(s)'</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>Column match: 'Virus name abbreviation(s)'</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>Column match: 'Virus isolate designation'</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>Column match: 'Virus GENBANK accession'</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>Column match: 'Genome coverage'</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>Column match: 'Genome'</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>Column match: 'Host source'</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>Column match: 'Accessions Link'</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>Column match: 'Editor Notes'</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>Column match: 'QC_status'</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>Column match: 'QC_taxon_inher_molecule'</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>Column match: 'QC_taxon_change'</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>Column match: 'QC_taxon_proposal'</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>Populating Original worksheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>Wrote 17916 rows into worksheet 'Original'</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>Populating VMR MSL40 worksheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>Wrote 17916 rows into worksheet 'VMR MSL40'</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>Added 17916 isolate hyperlinks in worksheet 'VMR MSL40'</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>Read 40 rows from file test_data/export/ICTVdatabase/data/taxonomy_toc.utf8.txt</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>Wrote workbook with 8 worksheet(s) to test_out/export/VMR.editor.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
         <is>
           <t>Wrote 4 worksheet(s) to public file test_out/export/VMR.xlsx</t>
         </is>

</xml_diff>